<commit_message>
Encargados, instancias e indicadores transaccionales nuevos
- Fichas: encargado de compradores y de proveedores (Power BI) bajo el ID,
  instancia y orden por instancia. La vigencia sigue siendo la del panel.
- Se quitan avisos de "instancia anterior" y la nota de término obsoleta.
- Transacciones: regiones unificadas (16), organismos consolidados por
  institución, sector comprador, ticket promedio, promedios mensuales,
  OC por organismo, top tipos de producto y comunas.
- Detalle: catálogo, ofertas y monto por tamaño de empresa (Power BI).
- Excel regenerados con regiones normalizadas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/oc-mensuales/administracion-y-entrega-de-beneficios/abr-2025.xlsx
+++ b/docs/oc-mensuales/administracion-y-entrega-de-beneficios/abr-2025.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OC abr-2025" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="OC abr-2025" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -549,7 +549,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Región de Arica y Parinacota</t>
+          <t>Arica y Parinacota</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -610,7 +610,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región del Maule </t>
+          <t>Maule</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -671,7 +671,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región del Biobío </t>
+          <t>Biobío</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -732,7 +732,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -854,7 +854,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -915,7 +915,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -976,7 +976,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1098,7 +1098,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1159,7 +1159,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Región de Los Ríos</t>
+          <t>Los Ríos</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1220,7 +1220,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1281,7 +1281,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Región de Los Ríos</t>
+          <t>Los Ríos</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Región Aysén del General Carlos Ibáñez del Campo</t>
+          <t>Aysén</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1403,7 +1403,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Región Aysén del General Carlos Ibáñez del Campo</t>
+          <t>Aysén</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1464,7 +1464,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1525,7 +1525,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1586,7 +1586,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de la Araucanía </t>
+          <t>Araucanía</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1647,7 +1647,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región del Maule </t>
+          <t>Maule</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1708,7 +1708,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de los Lagos </t>
+          <t>Los Lagos</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1769,7 +1769,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Región de Los Ríos</t>
+          <t>Los Ríos</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1830,7 +1830,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región del Biobío </t>
+          <t>Biobío</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1891,7 +1891,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1952,7 +1952,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2013,7 +2013,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2074,7 +2074,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2135,7 +2135,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2196,7 +2196,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de los Lagos </t>
+          <t>Los Lagos</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2257,7 +2257,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Región del Libertador General Bernardo O´Higgins</t>
+          <t>O'Higgins</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2318,7 +2318,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Región de Los Ríos</t>
+          <t>Los Ríos</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2379,7 +2379,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2440,7 +2440,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Región de Arica y Parinacota</t>
+          <t>Arica y Parinacota</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2501,7 +2501,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Región de Los Ríos</t>
+          <t>Los Ríos</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2562,7 +2562,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región del Biobío </t>
+          <t>Biobío</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2623,7 +2623,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región del Biobío </t>
+          <t>Biobío</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2684,7 +2684,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Región del Libertador General Bernardo O´Higgins</t>
+          <t>O'Higgins</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2745,7 +2745,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2806,7 +2806,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región del Maule </t>
+          <t>Maule</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Antofagasta </t>
+          <t>Antofagasta</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -2928,7 +2928,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Tarapacá  </t>
+          <t>Tarapacá</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -2989,7 +2989,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Región del Libertador General Bernardo O´Higgins</t>
+          <t>O'Higgins</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -3050,7 +3050,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -3111,7 +3111,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -3172,7 +3172,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Atacama </t>
+          <t>Atacama</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -3233,7 +3233,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -3294,7 +3294,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región del Biobío </t>
+          <t>Biobío</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -3355,7 +3355,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -3416,7 +3416,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -3477,7 +3477,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -3538,7 +3538,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -3599,7 +3599,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región del Biobío </t>
+          <t>Biobío</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -3660,7 +3660,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -3721,7 +3721,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Antofagasta </t>
+          <t>Antofagasta</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -3782,7 +3782,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>Región del Libertador General Bernardo O´Higgins</t>
+          <t>O'Higgins</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -3843,7 +3843,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de los Lagos </t>
+          <t>Los Lagos</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -3904,7 +3904,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Región del Libertador General Bernardo O´Higgins</t>
+          <t>O'Higgins</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -3965,7 +3965,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Antofagasta </t>
+          <t>Antofagasta</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -4026,7 +4026,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -4087,7 +4087,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región del Maule </t>
+          <t>Maule</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -4148,7 +4148,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>Región del Libertador General Bernardo O´Higgins</t>
+          <t>O'Higgins</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -4209,7 +4209,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -4270,7 +4270,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -4331,7 +4331,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -4392,7 +4392,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>Región Aysén del General Carlos Ibáñez del Campo</t>
+          <t>Aysén</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -4453,7 +4453,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>Región de Los Ríos</t>
+          <t>Los Ríos</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -4514,7 +4514,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de los Lagos </t>
+          <t>Los Lagos</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -4575,7 +4575,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Coquimbo </t>
+          <t>Coquimbo</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -4636,7 +4636,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Atacama </t>
+          <t>Atacama</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -4697,7 +4697,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -4758,7 +4758,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de la Araucanía </t>
+          <t>Araucanía</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -4819,7 +4819,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>Región Aysén del General Carlos Ibáñez del Campo</t>
+          <t>Aysén</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -4880,7 +4880,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -4941,7 +4941,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -5002,7 +5002,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -5063,7 +5063,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -5124,7 +5124,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de los Lagos </t>
+          <t>Los Lagos</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -5185,7 +5185,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -5368,7 +5368,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -5429,7 +5429,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -5490,7 +5490,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -5551,7 +5551,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>Región del Libertador General Bernardo O´Higgins</t>
+          <t>O'Higgins</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -5612,7 +5612,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -5673,7 +5673,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -5734,7 +5734,7 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>Bío-Bío</t>
+          <t>Biobío</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -5795,7 +5795,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -5856,7 +5856,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -5917,7 +5917,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Atacama </t>
+          <t>Atacama</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -5978,7 +5978,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -6100,7 +6100,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -6161,7 +6161,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -6222,7 +6222,7 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de la Araucanía </t>
+          <t>Araucanía</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -6283,7 +6283,7 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -6344,7 +6344,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -6405,7 +6405,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>Región de Los Ríos</t>
+          <t>Los Ríos</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -6466,7 +6466,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -6527,7 +6527,7 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -6649,7 +6649,7 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de los Lagos </t>
+          <t>Los Lagos</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -6710,7 +6710,7 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -6771,7 +6771,7 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -6832,7 +6832,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Antofagasta </t>
+          <t>Antofagasta</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -6893,7 +6893,7 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -6954,7 +6954,7 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -7015,7 +7015,7 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de los Lagos </t>
+          <t>Los Lagos</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -7076,7 +7076,7 @@
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -7137,7 +7137,7 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>Región del Libertador General Bernardo O´Higgins</t>
+          <t>O'Higgins</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -7198,7 +7198,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Antofagasta </t>
+          <t>Antofagasta</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -7259,7 +7259,7 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región del Maule </t>
+          <t>Maule</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -7320,7 +7320,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -7381,7 +7381,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -7442,7 +7442,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>Región del Libertador General Bernardo O´Higgins</t>
+          <t>O'Higgins</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -7503,7 +7503,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -7564,7 +7564,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -7625,7 +7625,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -7686,7 +7686,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de la Araucanía </t>
+          <t>Araucanía</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
@@ -7747,7 +7747,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -7808,7 +7808,7 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -7869,7 +7869,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
@@ -7930,7 +7930,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -7991,7 +7991,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
@@ -8052,7 +8052,7 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
@@ -8113,7 +8113,7 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -8174,7 +8174,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>Región del Libertador General Bernardo O´Higgins</t>
+          <t>O'Higgins</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -8235,7 +8235,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Antofagasta </t>
+          <t>Antofagasta</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -8357,7 +8357,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>Bío-Bío</t>
+          <t>Biobío</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
@@ -8418,7 +8418,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -8479,7 +8479,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -8540,7 +8540,7 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>Región del Libertador General Bernardo O´Higgins</t>
+          <t>O'Higgins</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -8601,7 +8601,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región del Maule </t>
+          <t>Maule</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -8662,7 +8662,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -8723,7 +8723,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -8784,7 +8784,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -8845,7 +8845,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región del Biobío </t>
+          <t>Biobío</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
@@ -8906,7 +8906,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -8967,7 +8967,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -9028,7 +9028,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de la Araucanía </t>
+          <t>Araucanía</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -9089,7 +9089,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de la Araucanía </t>
+          <t>Araucanía</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
@@ -9150,7 +9150,7 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -9211,7 +9211,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
@@ -9272,7 +9272,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Atacama </t>
+          <t>Atacama</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -9333,7 +9333,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
@@ -9394,7 +9394,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>Región del Ñuble</t>
+          <t>Ñuble</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
@@ -9455,7 +9455,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -9516,7 +9516,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
@@ -9577,7 +9577,7 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Atacama </t>
+          <t>Atacama</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
@@ -9699,7 +9699,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Tarapacá  </t>
+          <t>Tarapacá</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
@@ -9760,7 +9760,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de los Lagos </t>
+          <t>Los Lagos</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
@@ -9821,7 +9821,7 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>Región del Libertador General Bernardo O´Higgins</t>
+          <t>O'Higgins</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
@@ -9882,7 +9882,7 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
@@ -9943,7 +9943,7 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -10004,7 +10004,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>Región del Libertador General Bernardo O´Higgins</t>
+          <t>O'Higgins</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -10065,7 +10065,7 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de los Lagos </t>
+          <t>Los Lagos</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -10126,7 +10126,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Coquimbo </t>
+          <t>Coquimbo</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -10187,7 +10187,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de los Lagos </t>
+          <t>Los Lagos</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
@@ -10248,7 +10248,7 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de los Lagos </t>
+          <t>Los Lagos</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
@@ -10309,7 +10309,7 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de los Lagos </t>
+          <t>Los Lagos</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -10370,7 +10370,7 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
@@ -10431,7 +10431,7 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
@@ -10492,7 +10492,7 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
@@ -10553,7 +10553,7 @@
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
@@ -10614,7 +10614,7 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -10675,7 +10675,7 @@
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
@@ -10736,7 +10736,7 @@
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Antofagasta </t>
+          <t>Antofagasta</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
@@ -10858,7 +10858,7 @@
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región del Maule </t>
+          <t>Maule</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
@@ -10919,7 +10919,7 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>Región Aysén del General Carlos Ibáñez del Campo</t>
+          <t>Aysén</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
@@ -10980,7 +10980,7 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>Región Aysén del General Carlos Ibáñez del Campo</t>
+          <t>Aysén</t>
         </is>
       </c>
       <c r="I173" t="inlineStr">
@@ -11102,7 +11102,7 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I175" t="inlineStr">
@@ -11163,7 +11163,7 @@
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región del Maule </t>
+          <t>Maule</t>
         </is>
       </c>
       <c r="I176" t="inlineStr">
@@ -11224,7 +11224,7 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I177" t="inlineStr">
@@ -11285,7 +11285,7 @@
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I178" t="inlineStr">
@@ -11346,7 +11346,7 @@
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>Región del Libertador General Bernardo O´Higgins</t>
+          <t>O'Higgins</t>
         </is>
       </c>
       <c r="I179" t="inlineStr">
@@ -11529,7 +11529,7 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
@@ -11590,7 +11590,7 @@
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Antofagasta </t>
+          <t>Antofagasta</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
@@ -11651,7 +11651,7 @@
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
@@ -11712,7 +11712,7 @@
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Tarapacá  </t>
+          <t>Tarapacá</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
@@ -11773,7 +11773,7 @@
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
@@ -11834,7 +11834,7 @@
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>Región Aysén del General Carlos Ibáñez del Campo</t>
+          <t>Aysén</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
@@ -11895,7 +11895,7 @@
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
@@ -11956,7 +11956,7 @@
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>Región de Los Ríos</t>
+          <t>Los Ríos</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
@@ -12017,7 +12017,7 @@
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
@@ -12078,7 +12078,7 @@
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
@@ -12139,7 +12139,7 @@
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de los Lagos </t>
+          <t>Los Lagos</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
@@ -12200,7 +12200,7 @@
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
@@ -12261,7 +12261,7 @@
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>Región del Ñuble</t>
+          <t>Ñuble</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
@@ -12322,7 +12322,7 @@
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
@@ -12383,7 +12383,7 @@
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región del Biobío </t>
+          <t>Biobío</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
@@ -12444,7 +12444,7 @@
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
@@ -12505,7 +12505,7 @@
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región del Maule </t>
+          <t>Maule</t>
         </is>
       </c>
       <c r="I198" t="inlineStr">
@@ -12566,7 +12566,7 @@
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de la Araucanía </t>
+          <t>Araucanía</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
@@ -12627,7 +12627,7 @@
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>Región del Ñuble</t>
+          <t>Ñuble</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
@@ -12688,7 +12688,7 @@
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>Región del Libertador General Bernardo O´Higgins</t>
+          <t>O'Higgins</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
@@ -12749,7 +12749,7 @@
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I202" t="inlineStr">
@@ -12810,7 +12810,7 @@
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Tarapacá  </t>
+          <t>Tarapacá</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
@@ -12871,7 +12871,7 @@
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
@@ -12932,7 +12932,7 @@
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de los Lagos </t>
+          <t>Los Lagos</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
@@ -12993,7 +12993,7 @@
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de los Lagos </t>
+          <t>Los Lagos</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">
@@ -13054,7 +13054,7 @@
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>Región Aysén del General Carlos Ibáñez del Campo</t>
+          <t>Aysén</t>
         </is>
       </c>
       <c r="I207" t="inlineStr">
@@ -13115,7 +13115,7 @@
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región del Biobío </t>
+          <t>Biobío</t>
         </is>
       </c>
       <c r="I208" t="inlineStr">
@@ -13176,7 +13176,7 @@
       </c>
       <c r="H209" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I209" t="inlineStr">
@@ -13237,7 +13237,7 @@
       </c>
       <c r="H210" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Antofagasta </t>
+          <t>Antofagasta</t>
         </is>
       </c>
       <c r="I210" t="inlineStr">
@@ -13298,7 +13298,7 @@
       </c>
       <c r="H211" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I211" t="inlineStr">
@@ -13359,7 +13359,7 @@
       </c>
       <c r="H212" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de los Lagos </t>
+          <t>Los Lagos</t>
         </is>
       </c>
       <c r="I212" t="inlineStr">
@@ -13420,7 +13420,7 @@
       </c>
       <c r="H213" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I213" t="inlineStr">
@@ -13481,7 +13481,7 @@
       </c>
       <c r="H214" t="inlineStr">
         <is>
-          <t>Región Aysén del General Carlos Ibáñez del Campo</t>
+          <t>Aysén</t>
         </is>
       </c>
       <c r="I214" t="inlineStr">
@@ -13542,7 +13542,7 @@
       </c>
       <c r="H215" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I215" t="inlineStr">
@@ -13603,7 +13603,7 @@
       </c>
       <c r="H216" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I216" t="inlineStr">
@@ -13664,7 +13664,7 @@
       </c>
       <c r="H217" t="inlineStr">
         <is>
-          <t>Región del Libertador General Bernardo O´Higgins</t>
+          <t>O'Higgins</t>
         </is>
       </c>
       <c r="I217" t="inlineStr">
@@ -13725,7 +13725,7 @@
       </c>
       <c r="H218" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I218" t="inlineStr">
@@ -13786,7 +13786,7 @@
       </c>
       <c r="H219" t="inlineStr">
         <is>
-          <t>Región Aysén del General Carlos Ibáñez del Campo</t>
+          <t>Aysén</t>
         </is>
       </c>
       <c r="I219" t="inlineStr">
@@ -13847,7 +13847,7 @@
       </c>
       <c r="H220" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I220" t="inlineStr">
@@ -13908,7 +13908,7 @@
       </c>
       <c r="H221" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I221" t="inlineStr">
@@ -13969,7 +13969,7 @@
       </c>
       <c r="H222" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I222" t="inlineStr">
@@ -14030,7 +14030,7 @@
       </c>
       <c r="H223" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Tarapacá  </t>
+          <t>Tarapacá</t>
         </is>
       </c>
       <c r="I223" t="inlineStr">
@@ -14091,7 +14091,7 @@
       </c>
       <c r="H224" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I224" t="inlineStr">
@@ -14213,7 +14213,7 @@
       </c>
       <c r="H226" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región del Maule </t>
+          <t>Maule</t>
         </is>
       </c>
       <c r="I226" t="inlineStr">
@@ -14274,7 +14274,7 @@
       </c>
       <c r="H227" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región del Biobío </t>
+          <t>Biobío</t>
         </is>
       </c>
       <c r="I227" t="inlineStr">
@@ -14335,7 +14335,7 @@
       </c>
       <c r="H228" t="inlineStr">
         <is>
-          <t>Región del Libertador General Bernardo O´Higgins</t>
+          <t>O'Higgins</t>
         </is>
       </c>
       <c r="I228" t="inlineStr">
@@ -14396,7 +14396,7 @@
       </c>
       <c r="H229" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I229" t="inlineStr">
@@ -14457,7 +14457,7 @@
       </c>
       <c r="H230" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I230" t="inlineStr">
@@ -14518,7 +14518,7 @@
       </c>
       <c r="H231" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región del Maule </t>
+          <t>Maule</t>
         </is>
       </c>
       <c r="I231" t="inlineStr">
@@ -14579,7 +14579,7 @@
       </c>
       <c r="H232" t="inlineStr">
         <is>
-          <t>Región Aysén del General Carlos Ibáñez del Campo</t>
+          <t>Aysén</t>
         </is>
       </c>
       <c r="I232" t="inlineStr">
@@ -14701,7 +14701,7 @@
       </c>
       <c r="H234" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I234" t="inlineStr">
@@ -14762,7 +14762,7 @@
       </c>
       <c r="H235" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región del Biobío </t>
+          <t>Biobío</t>
         </is>
       </c>
       <c r="I235" t="inlineStr">
@@ -14884,7 +14884,7 @@
       </c>
       <c r="H237" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I237" t="inlineStr">
@@ -14945,7 +14945,7 @@
       </c>
       <c r="H238" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I238" t="inlineStr">
@@ -15006,7 +15006,7 @@
       </c>
       <c r="H239" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I239" t="inlineStr">
@@ -15067,7 +15067,7 @@
       </c>
       <c r="H240" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de los Lagos </t>
+          <t>Los Lagos</t>
         </is>
       </c>
       <c r="I240" t="inlineStr">
@@ -15128,7 +15128,7 @@
       </c>
       <c r="H241" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región del Maule </t>
+          <t>Maule</t>
         </is>
       </c>
       <c r="I241" t="inlineStr">
@@ -15189,7 +15189,7 @@
       </c>
       <c r="H242" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región del Biobío </t>
+          <t>Biobío</t>
         </is>
       </c>
       <c r="I242" t="inlineStr">
@@ -15250,7 +15250,7 @@
       </c>
       <c r="H243" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I243" t="inlineStr">
@@ -15372,7 +15372,7 @@
       </c>
       <c r="H245" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de la Araucanía </t>
+          <t>Araucanía</t>
         </is>
       </c>
       <c r="I245" t="inlineStr">
@@ -15433,7 +15433,7 @@
       </c>
       <c r="H246" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de la Araucanía </t>
+          <t>Araucanía</t>
         </is>
       </c>
       <c r="I246" t="inlineStr">
@@ -15494,7 +15494,7 @@
       </c>
       <c r="H247" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I247" t="inlineStr">
@@ -15555,7 +15555,7 @@
       </c>
       <c r="H248" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I248" t="inlineStr">
@@ -15616,7 +15616,7 @@
       </c>
       <c r="H249" t="inlineStr">
         <is>
-          <t>Región del Libertador General Bernardo O´Higgins</t>
+          <t>O'Higgins</t>
         </is>
       </c>
       <c r="I249" t="inlineStr">
@@ -15677,7 +15677,7 @@
       </c>
       <c r="H250" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I250" t="inlineStr">
@@ -15738,7 +15738,7 @@
       </c>
       <c r="H251" t="inlineStr">
         <is>
-          <t>Región del Libertador General Bernardo O´Higgins</t>
+          <t>O'Higgins</t>
         </is>
       </c>
       <c r="I251" t="inlineStr">
@@ -15799,7 +15799,7 @@
       </c>
       <c r="H252" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de los Lagos </t>
+          <t>Los Lagos</t>
         </is>
       </c>
       <c r="I252" t="inlineStr">
@@ -15860,7 +15860,7 @@
       </c>
       <c r="H253" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I253" t="inlineStr">
@@ -15921,7 +15921,7 @@
       </c>
       <c r="H254" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I254" t="inlineStr">
@@ -15982,7 +15982,7 @@
       </c>
       <c r="H255" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I255" t="inlineStr">
@@ -16043,7 +16043,7 @@
       </c>
       <c r="H256" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I256" t="inlineStr">
@@ -16104,7 +16104,7 @@
       </c>
       <c r="H257" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I257" t="inlineStr">
@@ -16165,7 +16165,7 @@
       </c>
       <c r="H258" t="inlineStr">
         <is>
-          <t>Región del Ñuble</t>
+          <t>Ñuble</t>
         </is>
       </c>
       <c r="I258" t="inlineStr">
@@ -16226,7 +16226,7 @@
       </c>
       <c r="H259" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I259" t="inlineStr">
@@ -16287,7 +16287,7 @@
       </c>
       <c r="H260" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de los Lagos </t>
+          <t>Los Lagos</t>
         </is>
       </c>
       <c r="I260" t="inlineStr">
@@ -16348,7 +16348,7 @@
       </c>
       <c r="H261" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región del Biobío </t>
+          <t>Biobío</t>
         </is>
       </c>
       <c r="I261" t="inlineStr">
@@ -16409,7 +16409,7 @@
       </c>
       <c r="H262" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Atacama </t>
+          <t>Atacama</t>
         </is>
       </c>
       <c r="I262" t="inlineStr">
@@ -16470,7 +16470,7 @@
       </c>
       <c r="H263" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de la Araucanía </t>
+          <t>Araucanía</t>
         </is>
       </c>
       <c r="I263" t="inlineStr">
@@ -16531,7 +16531,7 @@
       </c>
       <c r="H264" t="inlineStr">
         <is>
-          <t>Región de Los Ríos</t>
+          <t>Los Ríos</t>
         </is>
       </c>
       <c r="I264" t="inlineStr">
@@ -16592,7 +16592,7 @@
       </c>
       <c r="H265" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I265" t="inlineStr">
@@ -16653,7 +16653,7 @@
       </c>
       <c r="H266" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de la Araucanía </t>
+          <t>Araucanía</t>
         </is>
       </c>
       <c r="I266" t="inlineStr">
@@ -16714,7 +16714,7 @@
       </c>
       <c r="H267" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de la Araucanía </t>
+          <t>Araucanía</t>
         </is>
       </c>
       <c r="I267" t="inlineStr">
@@ -16775,7 +16775,7 @@
       </c>
       <c r="H268" t="inlineStr">
         <is>
-          <t>Región de Los Ríos</t>
+          <t>Los Ríos</t>
         </is>
       </c>
       <c r="I268" t="inlineStr">
@@ -16836,7 +16836,7 @@
       </c>
       <c r="H269" t="inlineStr">
         <is>
-          <t>Región del Libertador General Bernardo O´Higgins</t>
+          <t>O'Higgins</t>
         </is>
       </c>
       <c r="I269" t="inlineStr">
@@ -16897,7 +16897,7 @@
       </c>
       <c r="H270" t="inlineStr">
         <is>
-          <t>Región Aysén del General Carlos Ibáñez del Campo</t>
+          <t>Aysén</t>
         </is>
       </c>
       <c r="I270" t="inlineStr">
@@ -16958,7 +16958,7 @@
       </c>
       <c r="H271" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de la Araucanía </t>
+          <t>Araucanía</t>
         </is>
       </c>
       <c r="I271" t="inlineStr">
@@ -17019,7 +17019,7 @@
       </c>
       <c r="H272" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I272" t="inlineStr">
@@ -17080,7 +17080,7 @@
       </c>
       <c r="H273" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región del Biobío </t>
+          <t>Biobío</t>
         </is>
       </c>
       <c r="I273" t="inlineStr">
@@ -17141,7 +17141,7 @@
       </c>
       <c r="H274" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I274" t="inlineStr">
@@ -17202,7 +17202,7 @@
       </c>
       <c r="H275" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I275" t="inlineStr">
@@ -17324,7 +17324,7 @@
       </c>
       <c r="H277" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de la Araucanía </t>
+          <t>Araucanía</t>
         </is>
       </c>
       <c r="I277" t="inlineStr">
@@ -17385,7 +17385,7 @@
       </c>
       <c r="H278" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región del Biobío </t>
+          <t>Biobío</t>
         </is>
       </c>
       <c r="I278" t="inlineStr">
@@ -17446,7 +17446,7 @@
       </c>
       <c r="H279" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Coquimbo </t>
+          <t>Coquimbo</t>
         </is>
       </c>
       <c r="I279" t="inlineStr">
@@ -17507,7 +17507,7 @@
       </c>
       <c r="H280" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I280" t="inlineStr">
@@ -17629,7 +17629,7 @@
       </c>
       <c r="H282" t="inlineStr">
         <is>
-          <t>Región de Los Ríos</t>
+          <t>Los Ríos</t>
         </is>
       </c>
       <c r="I282" t="inlineStr">
@@ -17690,7 +17690,7 @@
       </c>
       <c r="H283" t="inlineStr">
         <is>
-          <t>Región Aysén del General Carlos Ibáñez del Campo</t>
+          <t>Aysén</t>
         </is>
       </c>
       <c r="I283" t="inlineStr">
@@ -17751,7 +17751,7 @@
       </c>
       <c r="H284" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I284" t="inlineStr">
@@ -17812,7 +17812,7 @@
       </c>
       <c r="H285" t="inlineStr">
         <is>
-          <t>Región de Magallanes y de la Antártica</t>
+          <t>Magallanes</t>
         </is>
       </c>
       <c r="I285" t="inlineStr">
@@ -17873,7 +17873,7 @@
       </c>
       <c r="H286" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I286" t="inlineStr">
@@ -17934,7 +17934,7 @@
       </c>
       <c r="H287" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I287" t="inlineStr">
@@ -17995,7 +17995,7 @@
       </c>
       <c r="H288" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de los Lagos </t>
+          <t>Los Lagos</t>
         </is>
       </c>
       <c r="I288" t="inlineStr">
@@ -18056,7 +18056,7 @@
       </c>
       <c r="H289" t="inlineStr">
         <is>
-          <t>Región Aysén del General Carlos Ibáñez del Campo</t>
+          <t>Aysén</t>
         </is>
       </c>
       <c r="I289" t="inlineStr">
@@ -18117,7 +18117,7 @@
       </c>
       <c r="H290" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de la Araucanía </t>
+          <t>Araucanía</t>
         </is>
       </c>
       <c r="I290" t="inlineStr">
@@ -18178,7 +18178,7 @@
       </c>
       <c r="H291" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Antofagasta </t>
+          <t>Antofagasta</t>
         </is>
       </c>
       <c r="I291" t="inlineStr">
@@ -18239,7 +18239,7 @@
       </c>
       <c r="H292" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I292" t="inlineStr">
@@ -18300,7 +18300,7 @@
       </c>
       <c r="H293" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I293" t="inlineStr">
@@ -18361,7 +18361,7 @@
       </c>
       <c r="H294" t="inlineStr">
         <is>
-          <t>Región del Ñuble</t>
+          <t>Ñuble</t>
         </is>
       </c>
       <c r="I294" t="inlineStr">
@@ -18422,7 +18422,7 @@
       </c>
       <c r="H295" t="inlineStr">
         <is>
-          <t>Región del Libertador General Bernardo O´Higgins</t>
+          <t>O'Higgins</t>
         </is>
       </c>
       <c r="I295" t="inlineStr">
@@ -18483,7 +18483,7 @@
       </c>
       <c r="H296" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de los Lagos </t>
+          <t>Los Lagos</t>
         </is>
       </c>
       <c r="I296" t="inlineStr">
@@ -18544,7 +18544,7 @@
       </c>
       <c r="H297" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Antofagasta </t>
+          <t>Antofagasta</t>
         </is>
       </c>
       <c r="I297" t="inlineStr">
@@ -18605,7 +18605,7 @@
       </c>
       <c r="H298" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I298" t="inlineStr">
@@ -18666,7 +18666,7 @@
       </c>
       <c r="H299" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I299" t="inlineStr">
@@ -18727,7 +18727,7 @@
       </c>
       <c r="H300" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Tarapacá  </t>
+          <t>Tarapacá</t>
         </is>
       </c>
       <c r="I300" t="inlineStr">
@@ -18788,7 +18788,7 @@
       </c>
       <c r="H301" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I301" t="inlineStr">
@@ -18849,7 +18849,7 @@
       </c>
       <c r="H302" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I302" t="inlineStr">
@@ -18910,7 +18910,7 @@
       </c>
       <c r="H303" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región del Biobío </t>
+          <t>Biobío</t>
         </is>
       </c>
       <c r="I303" t="inlineStr">
@@ -18971,7 +18971,7 @@
       </c>
       <c r="H304" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I304" t="inlineStr">
@@ -19032,7 +19032,7 @@
       </c>
       <c r="H305" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I305" t="inlineStr">
@@ -19093,7 +19093,7 @@
       </c>
       <c r="H306" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I306" t="inlineStr">
@@ -19154,7 +19154,7 @@
       </c>
       <c r="H307" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I307" t="inlineStr">
@@ -19276,7 +19276,7 @@
       </c>
       <c r="H309" t="inlineStr">
         <is>
-          <t>Región del Libertador General Bernardo O´Higgins</t>
+          <t>O'Higgins</t>
         </is>
       </c>
       <c r="I309" t="inlineStr">
@@ -19337,7 +19337,7 @@
       </c>
       <c r="H310" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I310" t="inlineStr">
@@ -19398,7 +19398,7 @@
       </c>
       <c r="H311" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región del Maule </t>
+          <t>Maule</t>
         </is>
       </c>
       <c r="I311" t="inlineStr">
@@ -19459,7 +19459,7 @@
       </c>
       <c r="H312" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I312" t="inlineStr">
@@ -19520,7 +19520,7 @@
       </c>
       <c r="H313" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Antofagasta </t>
+          <t>Antofagasta</t>
         </is>
       </c>
       <c r="I313" t="inlineStr">
@@ -19581,7 +19581,7 @@
       </c>
       <c r="H314" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Antofagasta </t>
+          <t>Antofagasta</t>
         </is>
       </c>
       <c r="I314" t="inlineStr">
@@ -19642,7 +19642,7 @@
       </c>
       <c r="H315" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de la Araucanía </t>
+          <t>Araucanía</t>
         </is>
       </c>
       <c r="I315" t="inlineStr">
@@ -19703,7 +19703,7 @@
       </c>
       <c r="H316" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Atacama </t>
+          <t>Atacama</t>
         </is>
       </c>
       <c r="I316" t="inlineStr">
@@ -19764,7 +19764,7 @@
       </c>
       <c r="H317" t="inlineStr">
         <is>
-          <t>Región de Los Ríos</t>
+          <t>Los Ríos</t>
         </is>
       </c>
       <c r="I317" t="inlineStr">
@@ -19825,7 +19825,7 @@
       </c>
       <c r="H318" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región del Biobío </t>
+          <t>Biobío</t>
         </is>
       </c>
       <c r="I318" t="inlineStr">
@@ -19886,7 +19886,7 @@
       </c>
       <c r="H319" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I319" t="inlineStr">
@@ -19947,7 +19947,7 @@
       </c>
       <c r="H320" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I320" t="inlineStr">
@@ -20008,7 +20008,7 @@
       </c>
       <c r="H321" t="inlineStr">
         <is>
-          <t>Región del Libertador General Bernardo O´Higgins</t>
+          <t>O'Higgins</t>
         </is>
       </c>
       <c r="I321" t="inlineStr">
@@ -20069,7 +20069,7 @@
       </c>
       <c r="H322" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Atacama </t>
+          <t>Atacama</t>
         </is>
       </c>
       <c r="I322" t="inlineStr">
@@ -20130,7 +20130,7 @@
       </c>
       <c r="H323" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I323" t="inlineStr">
@@ -20191,7 +20191,7 @@
       </c>
       <c r="H324" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I324" t="inlineStr">
@@ -20252,7 +20252,7 @@
       </c>
       <c r="H325" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de los Lagos </t>
+          <t>Los Lagos</t>
         </is>
       </c>
       <c r="I325" t="inlineStr">
@@ -20313,7 +20313,7 @@
       </c>
       <c r="H326" t="inlineStr">
         <is>
-          <t>Magallanes y Antártica</t>
+          <t>Magallanes</t>
         </is>
       </c>
       <c r="I326" t="inlineStr">
@@ -20374,7 +20374,7 @@
       </c>
       <c r="H327" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de la Araucanía </t>
+          <t>Araucanía</t>
         </is>
       </c>
       <c r="I327" t="inlineStr">
@@ -20435,7 +20435,7 @@
       </c>
       <c r="H328" t="inlineStr">
         <is>
-          <t>Región del Libertador General Bernardo O´Higgins</t>
+          <t>O'Higgins</t>
         </is>
       </c>
       <c r="I328" t="inlineStr">
@@ -20496,7 +20496,7 @@
       </c>
       <c r="H329" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de la Araucanía </t>
+          <t>Araucanía</t>
         </is>
       </c>
       <c r="I329" t="inlineStr">
@@ -20557,7 +20557,7 @@
       </c>
       <c r="H330" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región del Maule </t>
+          <t>Maule</t>
         </is>
       </c>
       <c r="I330" t="inlineStr">
@@ -20618,7 +20618,7 @@
       </c>
       <c r="H331" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I331" t="inlineStr">
@@ -20679,7 +20679,7 @@
       </c>
       <c r="H332" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de los Lagos </t>
+          <t>Los Lagos</t>
         </is>
       </c>
       <c r="I332" t="inlineStr">
@@ -20740,7 +20740,7 @@
       </c>
       <c r="H333" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región del Biobío </t>
+          <t>Biobío</t>
         </is>
       </c>
       <c r="I333" t="inlineStr">
@@ -20862,7 +20862,7 @@
       </c>
       <c r="H335" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I335" t="inlineStr">
@@ -20923,7 +20923,7 @@
       </c>
       <c r="H336" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región del Biobío </t>
+          <t>Biobío</t>
         </is>
       </c>
       <c r="I336" t="inlineStr">
@@ -20984,7 +20984,7 @@
       </c>
       <c r="H337" t="inlineStr">
         <is>
-          <t>Región del Libertador General Bernardo O´Higgins</t>
+          <t>O'Higgins</t>
         </is>
       </c>
       <c r="I337" t="inlineStr">
@@ -21045,7 +21045,7 @@
       </c>
       <c r="H338" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región del Maule </t>
+          <t>Maule</t>
         </is>
       </c>
       <c r="I338" t="inlineStr">
@@ -21106,7 +21106,7 @@
       </c>
       <c r="H339" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de la Araucanía </t>
+          <t>Araucanía</t>
         </is>
       </c>
       <c r="I339" t="inlineStr">
@@ -21167,7 +21167,7 @@
       </c>
       <c r="H340" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I340" t="inlineStr">
@@ -21228,7 +21228,7 @@
       </c>
       <c r="H341" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I341" t="inlineStr">
@@ -21289,7 +21289,7 @@
       </c>
       <c r="H342" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de la Araucanía </t>
+          <t>Araucanía</t>
         </is>
       </c>
       <c r="I342" t="inlineStr">
@@ -21411,7 +21411,7 @@
       </c>
       <c r="H344" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región del Maule </t>
+          <t>Maule</t>
         </is>
       </c>
       <c r="I344" t="inlineStr">
@@ -21472,7 +21472,7 @@
       </c>
       <c r="H345" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I345" t="inlineStr">
@@ -21533,7 +21533,7 @@
       </c>
       <c r="H346" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región del Biobío </t>
+          <t>Biobío</t>
         </is>
       </c>
       <c r="I346" t="inlineStr">
@@ -21594,7 +21594,7 @@
       </c>
       <c r="H347" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región del Biobío </t>
+          <t>Biobío</t>
         </is>
       </c>
       <c r="I347" t="inlineStr">
@@ -21655,7 +21655,7 @@
       </c>
       <c r="H348" t="inlineStr">
         <is>
-          <t>Región de Magallanes y de la Antártica</t>
+          <t>Magallanes</t>
         </is>
       </c>
       <c r="I348" t="inlineStr">
@@ -21716,7 +21716,7 @@
       </c>
       <c r="H349" t="inlineStr">
         <is>
-          <t>Región Aysén del General Carlos Ibáñez del Campo</t>
+          <t>Aysén</t>
         </is>
       </c>
       <c r="I349" t="inlineStr">
@@ -21777,7 +21777,7 @@
       </c>
       <c r="H350" t="inlineStr">
         <is>
-          <t>Región de Magallanes y de la Antártica</t>
+          <t>Magallanes</t>
         </is>
       </c>
       <c r="I350" t="inlineStr">
@@ -21838,7 +21838,7 @@
       </c>
       <c r="H351" t="inlineStr">
         <is>
-          <t>Región del Ñuble</t>
+          <t>Ñuble</t>
         </is>
       </c>
       <c r="I351" t="inlineStr">
@@ -21960,7 +21960,7 @@
       </c>
       <c r="H353" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I353" t="inlineStr">
@@ -22021,7 +22021,7 @@
       </c>
       <c r="H354" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I354" t="inlineStr">
@@ -22143,7 +22143,7 @@
       </c>
       <c r="H356" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región del Maule </t>
+          <t>Maule</t>
         </is>
       </c>
       <c r="I356" t="inlineStr">
@@ -22204,7 +22204,7 @@
       </c>
       <c r="H357" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región del Maule </t>
+          <t>Maule</t>
         </is>
       </c>
       <c r="I357" t="inlineStr">
@@ -22265,7 +22265,7 @@
       </c>
       <c r="H358" t="inlineStr">
         <is>
-          <t>Región de Magallanes y de la Antártica</t>
+          <t>Magallanes</t>
         </is>
       </c>
       <c r="I358" t="inlineStr">
@@ -22387,7 +22387,7 @@
       </c>
       <c r="H360" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de la Araucanía </t>
+          <t>Araucanía</t>
         </is>
       </c>
       <c r="I360" t="inlineStr">
@@ -22448,7 +22448,7 @@
       </c>
       <c r="H361" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de la Araucanía </t>
+          <t>Araucanía</t>
         </is>
       </c>
       <c r="I361" t="inlineStr">
@@ -22509,7 +22509,7 @@
       </c>
       <c r="H362" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I362" t="inlineStr">
@@ -22570,7 +22570,7 @@
       </c>
       <c r="H363" t="inlineStr">
         <is>
-          <t>Región del Ñuble</t>
+          <t>Ñuble</t>
         </is>
       </c>
       <c r="I363" t="inlineStr">
@@ -22631,7 +22631,7 @@
       </c>
       <c r="H364" t="inlineStr">
         <is>
-          <t>Región del Libertador General Bernardo O´Higgins</t>
+          <t>O'Higgins</t>
         </is>
       </c>
       <c r="I364" t="inlineStr">
@@ -22692,7 +22692,7 @@
       </c>
       <c r="H365" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región del Maule </t>
+          <t>Maule</t>
         </is>
       </c>
       <c r="I365" t="inlineStr">
@@ -22753,7 +22753,7 @@
       </c>
       <c r="H366" t="inlineStr">
         <is>
-          <t>Región del Ñuble</t>
+          <t>Ñuble</t>
         </is>
       </c>
       <c r="I366" t="inlineStr">
@@ -22814,7 +22814,7 @@
       </c>
       <c r="H367" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I367" t="inlineStr">
@@ -22875,7 +22875,7 @@
       </c>
       <c r="H368" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I368" t="inlineStr">
@@ -22936,7 +22936,7 @@
       </c>
       <c r="H369" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I369" t="inlineStr">
@@ -22997,7 +22997,7 @@
       </c>
       <c r="H370" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I370" t="inlineStr">
@@ -23058,7 +23058,7 @@
       </c>
       <c r="H371" t="inlineStr">
         <is>
-          <t>Región Aysén del General Carlos Ibáñez del Campo</t>
+          <t>Aysén</t>
         </is>
       </c>
       <c r="I371" t="inlineStr">
@@ -23180,7 +23180,7 @@
       </c>
       <c r="H373" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de los Lagos </t>
+          <t>Los Lagos</t>
         </is>
       </c>
       <c r="I373" t="inlineStr">
@@ -23241,7 +23241,7 @@
       </c>
       <c r="H374" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I374" t="inlineStr">
@@ -23302,7 +23302,7 @@
       </c>
       <c r="H375" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I375" t="inlineStr">
@@ -23363,7 +23363,7 @@
       </c>
       <c r="H376" t="inlineStr">
         <is>
-          <t>Región Aysén del General Carlos Ibáñez del Campo</t>
+          <t>Aysén</t>
         </is>
       </c>
       <c r="I376" t="inlineStr">
@@ -23424,7 +23424,7 @@
       </c>
       <c r="H377" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I377" t="inlineStr">
@@ -23485,7 +23485,7 @@
       </c>
       <c r="H378" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de Valparaíso </t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I378" t="inlineStr">
@@ -23546,7 +23546,7 @@
       </c>
       <c r="H379" t="inlineStr">
         <is>
-          <t>Región de Arica y Parinacota</t>
+          <t>Arica y Parinacota</t>
         </is>
       </c>
       <c r="I379" t="inlineStr">
@@ -23607,7 +23607,7 @@
       </c>
       <c r="H380" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región del Maule </t>
+          <t>Maule</t>
         </is>
       </c>
       <c r="I380" t="inlineStr">
@@ -23668,7 +23668,7 @@
       </c>
       <c r="H381" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I381" t="inlineStr">
@@ -23729,7 +23729,7 @@
       </c>
       <c r="H382" t="inlineStr">
         <is>
-          <t xml:space="preserve">Región de la Araucanía </t>
+          <t>Araucanía</t>
         </is>
       </c>
       <c r="I382" t="inlineStr">
@@ -23790,7 +23790,7 @@
       </c>
       <c r="H383" t="inlineStr">
         <is>
-          <t>Región del Libertador General Bernardo O´Higgins</t>
+          <t>O'Higgins</t>
         </is>
       </c>
       <c r="I383" t="inlineStr">
@@ -23851,7 +23851,7 @@
       </c>
       <c r="H384" t="inlineStr">
         <is>
-          <t>Región Metropolitana de Santiago</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I384" t="inlineStr">

</xml_diff>

<commit_message>
Completa datos transaccionales con la base de OC 2025-2026
- Incluye convenios anteriores de Alimentos (2239-7-LR17), Gas (2239-6-LR23)
  y Escritorio (2239-2-LR23), con nota y IDs en el detalle.
- OC SE/CC sin código: se recupera la licitación cuando está escrita en el
  texto de la OC (95% de coincidencia con Datos Abiertos).
- Región del proveedor completada desde su comuna (75% de las OC).
- Se excluye la OC 1395481-9-SE25 (7,3 millones de UF), monto inverosímil.
- Notas de licitaciones anteriores en todos los convenios que las tienen.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/oc-mensuales/administracion-y-entrega-de-beneficios/abr-2025.xlsx
+++ b/docs/oc-mensuales/administracion-y-entrega-de-beneficios/abr-2025.xlsx
@@ -562,7 +562,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L2" t="inlineStr">
         <is>
           <t>USD</t>
@@ -623,7 +627,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L3" t="inlineStr">
         <is>
           <t>USD</t>
@@ -684,7 +692,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L4" t="inlineStr">
         <is>
           <t>USD</t>
@@ -745,7 +757,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L5" t="inlineStr">
         <is>
           <t>USD</t>
@@ -806,7 +822,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L6" t="inlineStr">
         <is>
           <t>USD</t>
@@ -867,7 +887,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L7" t="inlineStr">
         <is>
           <t>USD</t>
@@ -928,7 +952,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L8" t="inlineStr">
         <is>
           <t>USD</t>
@@ -989,7 +1017,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L9" t="inlineStr">
         <is>
           <t>USD</t>
@@ -1050,7 +1082,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L10" t="inlineStr">
         <is>
           <t>USD</t>
@@ -1111,7 +1147,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr"/>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L11" t="inlineStr">
         <is>
           <t>USD</t>
@@ -1172,7 +1212,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr"/>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L12" t="inlineStr">
         <is>
           <t>USD</t>
@@ -1233,7 +1277,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr"/>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L13" t="inlineStr">
         <is>
           <t>USD</t>
@@ -1294,7 +1342,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr"/>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L14" t="inlineStr">
         <is>
           <t>USD</t>
@@ -1355,7 +1407,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr"/>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L15" t="inlineStr">
         <is>
           <t>USD</t>
@@ -1416,7 +1472,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr"/>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L16" t="inlineStr">
         <is>
           <t>USD</t>
@@ -1477,7 +1537,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr"/>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L17" t="inlineStr">
         <is>
           <t>USD</t>
@@ -1538,7 +1602,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr"/>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L18" t="inlineStr">
         <is>
           <t>USD</t>
@@ -1599,7 +1667,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr"/>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L19" t="inlineStr">
         <is>
           <t>USD</t>
@@ -1660,7 +1732,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr"/>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L20" t="inlineStr">
         <is>
           <t>USD</t>
@@ -1721,7 +1797,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr"/>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L21" t="inlineStr">
         <is>
           <t>USD</t>
@@ -1782,7 +1862,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr"/>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L22" t="inlineStr">
         <is>
           <t>USD</t>
@@ -1843,7 +1927,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr"/>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L23" t="inlineStr">
         <is>
           <t>USD</t>
@@ -1904,7 +1992,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr"/>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L24" t="inlineStr">
         <is>
           <t>USD</t>
@@ -1965,7 +2057,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr"/>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L25" t="inlineStr">
         <is>
           <t>USD</t>
@@ -2026,7 +2122,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr"/>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L26" t="inlineStr">
         <is>
           <t>USD</t>
@@ -2087,7 +2187,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr"/>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L27" t="inlineStr">
         <is>
           <t>USD</t>
@@ -2148,7 +2252,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr"/>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L28" t="inlineStr">
         <is>
           <t>USD</t>
@@ -2209,7 +2317,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr"/>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L29" t="inlineStr">
         <is>
           <t>USD</t>
@@ -2270,7 +2382,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr"/>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L30" t="inlineStr">
         <is>
           <t>USD</t>
@@ -2331,7 +2447,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr"/>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L31" t="inlineStr">
         <is>
           <t>USD</t>
@@ -2392,7 +2512,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr"/>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L32" t="inlineStr">
         <is>
           <t>USD</t>
@@ -2453,7 +2577,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr"/>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L33" t="inlineStr">
         <is>
           <t>USD</t>
@@ -2514,7 +2642,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr"/>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L34" t="inlineStr">
         <is>
           <t>USD</t>
@@ -2575,7 +2707,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr"/>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L35" t="inlineStr">
         <is>
           <t>USD</t>
@@ -2636,7 +2772,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr"/>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L36" t="inlineStr">
         <is>
           <t>USD</t>
@@ -2697,7 +2837,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K37" t="inlineStr"/>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L37" t="inlineStr">
         <is>
           <t>USD</t>
@@ -2758,7 +2902,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr"/>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L38" t="inlineStr">
         <is>
           <t>USD</t>
@@ -2819,7 +2967,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr"/>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L39" t="inlineStr">
         <is>
           <t>USD</t>
@@ -2880,7 +3032,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr"/>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L40" t="inlineStr">
         <is>
           <t>USD</t>
@@ -2941,7 +3097,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr"/>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L41" t="inlineStr">
         <is>
           <t>USD</t>
@@ -3002,7 +3162,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr"/>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L42" t="inlineStr">
         <is>
           <t>USD</t>
@@ -3063,7 +3227,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr"/>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L43" t="inlineStr">
         <is>
           <t>USD</t>
@@ -3124,7 +3292,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr"/>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L44" t="inlineStr">
         <is>
           <t>USD</t>
@@ -3185,7 +3357,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr"/>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L45" t="inlineStr">
         <is>
           <t>USD</t>
@@ -3246,7 +3422,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr"/>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L46" t="inlineStr">
         <is>
           <t>USD</t>
@@ -3307,7 +3487,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr"/>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L47" t="inlineStr">
         <is>
           <t>USD</t>
@@ -3368,7 +3552,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K48" t="inlineStr"/>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L48" t="inlineStr">
         <is>
           <t>USD</t>
@@ -3429,7 +3617,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr"/>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L49" t="inlineStr">
         <is>
           <t>USD</t>
@@ -3490,7 +3682,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr"/>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L50" t="inlineStr">
         <is>
           <t>USD</t>
@@ -3551,7 +3747,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K51" t="inlineStr"/>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L51" t="inlineStr">
         <is>
           <t>USD</t>
@@ -3612,7 +3812,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr"/>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L52" t="inlineStr">
         <is>
           <t>USD</t>
@@ -3673,7 +3877,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K53" t="inlineStr"/>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L53" t="inlineStr">
         <is>
           <t>USD</t>
@@ -3734,7 +3942,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K54" t="inlineStr"/>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L54" t="inlineStr">
         <is>
           <t>USD</t>
@@ -3795,7 +4007,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K55" t="inlineStr"/>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L55" t="inlineStr">
         <is>
           <t>USD</t>
@@ -3856,7 +4072,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K56" t="inlineStr"/>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L56" t="inlineStr">
         <is>
           <t>USD</t>
@@ -3917,7 +4137,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K57" t="inlineStr"/>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L57" t="inlineStr">
         <is>
           <t>USD</t>
@@ -3978,7 +4202,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K58" t="inlineStr"/>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L58" t="inlineStr">
         <is>
           <t>USD</t>
@@ -4039,7 +4267,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K59" t="inlineStr"/>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L59" t="inlineStr">
         <is>
           <t>USD</t>
@@ -4100,7 +4332,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K60" t="inlineStr"/>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L60" t="inlineStr">
         <is>
           <t>USD</t>
@@ -4161,7 +4397,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K61" t="inlineStr"/>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L61" t="inlineStr">
         <is>
           <t>USD</t>
@@ -4222,7 +4462,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K62" t="inlineStr"/>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L62" t="inlineStr">
         <is>
           <t>USD</t>
@@ -4283,7 +4527,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K63" t="inlineStr"/>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L63" t="inlineStr">
         <is>
           <t>USD</t>
@@ -4344,7 +4592,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K64" t="inlineStr"/>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L64" t="inlineStr">
         <is>
           <t>USD</t>
@@ -4405,7 +4657,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K65" t="inlineStr"/>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L65" t="inlineStr">
         <is>
           <t>USD</t>
@@ -4466,7 +4722,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K66" t="inlineStr"/>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L66" t="inlineStr">
         <is>
           <t>USD</t>
@@ -4527,7 +4787,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K67" t="inlineStr"/>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L67" t="inlineStr">
         <is>
           <t>USD</t>
@@ -4588,7 +4852,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K68" t="inlineStr"/>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L68" t="inlineStr">
         <is>
           <t>USD</t>
@@ -4649,7 +4917,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K69" t="inlineStr"/>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L69" t="inlineStr">
         <is>
           <t>USD</t>
@@ -4710,7 +4982,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K70" t="inlineStr"/>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L70" t="inlineStr">
         <is>
           <t>USD</t>
@@ -4771,7 +5047,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K71" t="inlineStr"/>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L71" t="inlineStr">
         <is>
           <t>USD</t>
@@ -4832,7 +5112,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K72" t="inlineStr"/>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L72" t="inlineStr">
         <is>
           <t>USD</t>
@@ -4893,7 +5177,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K73" t="inlineStr"/>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L73" t="inlineStr">
         <is>
           <t>USD</t>
@@ -4954,7 +5242,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K74" t="inlineStr"/>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L74" t="inlineStr">
         <is>
           <t>USD</t>
@@ -5015,7 +5307,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K75" t="inlineStr"/>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L75" t="inlineStr">
         <is>
           <t>USD</t>
@@ -5076,7 +5372,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K76" t="inlineStr"/>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L76" t="inlineStr">
         <is>
           <t>USD</t>
@@ -5137,7 +5437,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K77" t="inlineStr"/>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L77" t="inlineStr">
         <is>
           <t>USD</t>
@@ -5198,7 +5502,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K78" t="inlineStr"/>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L78" t="inlineStr">
         <is>
           <t>USD</t>
@@ -5259,7 +5567,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K79" t="inlineStr"/>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L79" t="inlineStr">
         <is>
           <t>USD</t>
@@ -5320,7 +5632,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K80" t="inlineStr"/>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L80" t="inlineStr">
         <is>
           <t>USD</t>
@@ -5381,7 +5697,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K81" t="inlineStr"/>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L81" t="inlineStr">
         <is>
           <t>USD</t>
@@ -5442,7 +5762,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K82" t="inlineStr"/>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L82" t="inlineStr">
         <is>
           <t>USD</t>
@@ -5503,7 +5827,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K83" t="inlineStr"/>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L83" t="inlineStr">
         <is>
           <t>USD</t>
@@ -5564,7 +5892,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K84" t="inlineStr"/>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L84" t="inlineStr">
         <is>
           <t>USD</t>
@@ -5625,7 +5957,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K85" t="inlineStr"/>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L85" t="inlineStr">
         <is>
           <t>USD</t>
@@ -5686,7 +6022,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K86" t="inlineStr"/>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L86" t="inlineStr">
         <is>
           <t>USD</t>
@@ -5747,7 +6087,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K87" t="inlineStr"/>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L87" t="inlineStr">
         <is>
           <t>USD</t>
@@ -5808,7 +6152,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K88" t="inlineStr"/>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L88" t="inlineStr">
         <is>
           <t>USD</t>
@@ -5869,7 +6217,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K89" t="inlineStr"/>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L89" t="inlineStr">
         <is>
           <t>USD</t>
@@ -5930,7 +6282,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K90" t="inlineStr"/>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L90" t="inlineStr">
         <is>
           <t>USD</t>
@@ -5991,7 +6347,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K91" t="inlineStr"/>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L91" t="inlineStr">
         <is>
           <t>USD</t>
@@ -6052,7 +6412,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K92" t="inlineStr"/>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L92" t="inlineStr">
         <is>
           <t>USD</t>
@@ -6113,7 +6477,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K93" t="inlineStr"/>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L93" t="inlineStr">
         <is>
           <t>USD</t>
@@ -6174,7 +6542,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K94" t="inlineStr"/>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L94" t="inlineStr">
         <is>
           <t>USD</t>
@@ -6235,7 +6607,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K95" t="inlineStr"/>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L95" t="inlineStr">
         <is>
           <t>USD</t>
@@ -6296,7 +6672,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K96" t="inlineStr"/>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L96" t="inlineStr">
         <is>
           <t>USD</t>
@@ -6357,7 +6737,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K97" t="inlineStr"/>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L97" t="inlineStr">
         <is>
           <t>USD</t>
@@ -6418,7 +6802,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K98" t="inlineStr"/>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L98" t="inlineStr">
         <is>
           <t>USD</t>
@@ -6479,7 +6867,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K99" t="inlineStr"/>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L99" t="inlineStr">
         <is>
           <t>USD</t>
@@ -6540,7 +6932,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K100" t="inlineStr"/>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L100" t="inlineStr">
         <is>
           <t>USD</t>
@@ -6601,7 +6997,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K101" t="inlineStr"/>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L101" t="inlineStr">
         <is>
           <t>USD</t>
@@ -6662,7 +7062,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K102" t="inlineStr"/>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L102" t="inlineStr">
         <is>
           <t>USD</t>
@@ -6723,7 +7127,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K103" t="inlineStr"/>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L103" t="inlineStr">
         <is>
           <t>USD</t>
@@ -6784,7 +7192,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K104" t="inlineStr"/>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L104" t="inlineStr">
         <is>
           <t>USD</t>
@@ -6845,7 +7257,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K105" t="inlineStr"/>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L105" t="inlineStr">
         <is>
           <t>USD</t>
@@ -6906,7 +7322,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K106" t="inlineStr"/>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L106" t="inlineStr">
         <is>
           <t>USD</t>
@@ -6967,7 +7387,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K107" t="inlineStr"/>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L107" t="inlineStr">
         <is>
           <t>USD</t>
@@ -7028,7 +7452,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K108" t="inlineStr"/>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L108" t="inlineStr">
         <is>
           <t>USD</t>
@@ -7089,7 +7517,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K109" t="inlineStr"/>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L109" t="inlineStr">
         <is>
           <t>USD</t>
@@ -7150,7 +7582,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K110" t="inlineStr"/>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L110" t="inlineStr">
         <is>
           <t>USD</t>
@@ -7211,7 +7647,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K111" t="inlineStr"/>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L111" t="inlineStr">
         <is>
           <t>USD</t>
@@ -7272,7 +7712,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K112" t="inlineStr"/>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L112" t="inlineStr">
         <is>
           <t>USD</t>
@@ -7333,7 +7777,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K113" t="inlineStr"/>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L113" t="inlineStr">
         <is>
           <t>USD</t>
@@ -7394,7 +7842,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K114" t="inlineStr"/>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L114" t="inlineStr">
         <is>
           <t>USD</t>
@@ -7455,7 +7907,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K115" t="inlineStr"/>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L115" t="inlineStr">
         <is>
           <t>USD</t>
@@ -7516,7 +7972,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K116" t="inlineStr"/>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L116" t="inlineStr">
         <is>
           <t>USD</t>
@@ -7577,7 +8037,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K117" t="inlineStr"/>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L117" t="inlineStr">
         <is>
           <t>USD</t>
@@ -7638,7 +8102,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K118" t="inlineStr"/>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L118" t="inlineStr">
         <is>
           <t>USD</t>
@@ -7699,7 +8167,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K119" t="inlineStr"/>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L119" t="inlineStr">
         <is>
           <t>USD</t>
@@ -7760,7 +8232,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K120" t="inlineStr"/>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L120" t="inlineStr">
         <is>
           <t>USD</t>
@@ -7821,7 +8297,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K121" t="inlineStr"/>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L121" t="inlineStr">
         <is>
           <t>USD</t>
@@ -7882,7 +8362,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K122" t="inlineStr"/>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L122" t="inlineStr">
         <is>
           <t>USD</t>
@@ -7943,7 +8427,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K123" t="inlineStr"/>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L123" t="inlineStr">
         <is>
           <t>USD</t>
@@ -8004,7 +8492,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K124" t="inlineStr"/>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L124" t="inlineStr">
         <is>
           <t>USD</t>
@@ -8065,7 +8557,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K125" t="inlineStr"/>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L125" t="inlineStr">
         <is>
           <t>USD</t>
@@ -8126,7 +8622,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K126" t="inlineStr"/>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L126" t="inlineStr">
         <is>
           <t>USD</t>
@@ -8187,7 +8687,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K127" t="inlineStr"/>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L127" t="inlineStr">
         <is>
           <t>USD</t>
@@ -8248,7 +8752,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K128" t="inlineStr"/>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L128" t="inlineStr">
         <is>
           <t>USD</t>
@@ -8309,7 +8817,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K129" t="inlineStr"/>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L129" t="inlineStr">
         <is>
           <t>USD</t>
@@ -8370,7 +8882,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K130" t="inlineStr"/>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L130" t="inlineStr">
         <is>
           <t>USD</t>
@@ -8431,7 +8947,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K131" t="inlineStr"/>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L131" t="inlineStr">
         <is>
           <t>USD</t>
@@ -8492,7 +9012,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K132" t="inlineStr"/>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L132" t="inlineStr">
         <is>
           <t>USD</t>
@@ -8553,7 +9077,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K133" t="inlineStr"/>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L133" t="inlineStr">
         <is>
           <t>USD</t>
@@ -8614,7 +9142,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K134" t="inlineStr"/>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L134" t="inlineStr">
         <is>
           <t>USD</t>
@@ -8675,7 +9207,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K135" t="inlineStr"/>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L135" t="inlineStr">
         <is>
           <t>USD</t>
@@ -8736,7 +9272,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K136" t="inlineStr"/>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L136" t="inlineStr">
         <is>
           <t>USD</t>
@@ -8797,7 +9337,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K137" t="inlineStr"/>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L137" t="inlineStr">
         <is>
           <t>USD</t>
@@ -8858,7 +9402,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K138" t="inlineStr"/>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L138" t="inlineStr">
         <is>
           <t>USD</t>
@@ -8919,7 +9467,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K139" t="inlineStr"/>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L139" t="inlineStr">
         <is>
           <t>USD</t>
@@ -8980,7 +9532,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K140" t="inlineStr"/>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L140" t="inlineStr">
         <is>
           <t>USD</t>
@@ -9041,7 +9597,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K141" t="inlineStr"/>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L141" t="inlineStr">
         <is>
           <t>USD</t>
@@ -9102,7 +9662,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K142" t="inlineStr"/>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L142" t="inlineStr">
         <is>
           <t>USD</t>
@@ -9163,7 +9727,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K143" t="inlineStr"/>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L143" t="inlineStr">
         <is>
           <t>USD</t>
@@ -9224,7 +9792,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K144" t="inlineStr"/>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L144" t="inlineStr">
         <is>
           <t>USD</t>
@@ -9285,7 +9857,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K145" t="inlineStr"/>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L145" t="inlineStr">
         <is>
           <t>USD</t>
@@ -9346,7 +9922,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K146" t="inlineStr"/>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L146" t="inlineStr">
         <is>
           <t>USD</t>
@@ -9407,7 +9987,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K147" t="inlineStr"/>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L147" t="inlineStr">
         <is>
           <t>USD</t>
@@ -9468,7 +10052,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K148" t="inlineStr"/>
+      <c r="K148" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L148" t="inlineStr">
         <is>
           <t>USD</t>
@@ -9529,7 +10117,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K149" t="inlineStr"/>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L149" t="inlineStr">
         <is>
           <t>USD</t>
@@ -9590,7 +10182,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K150" t="inlineStr"/>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L150" t="inlineStr">
         <is>
           <t>USD</t>
@@ -9651,7 +10247,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K151" t="inlineStr"/>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L151" t="inlineStr">
         <is>
           <t>USD</t>
@@ -9712,7 +10312,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K152" t="inlineStr"/>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L152" t="inlineStr">
         <is>
           <t>USD</t>
@@ -9773,7 +10377,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K153" t="inlineStr"/>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L153" t="inlineStr">
         <is>
           <t>USD</t>
@@ -9834,7 +10442,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K154" t="inlineStr"/>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L154" t="inlineStr">
         <is>
           <t>USD</t>
@@ -9895,7 +10507,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K155" t="inlineStr"/>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L155" t="inlineStr">
         <is>
           <t>USD</t>
@@ -9956,7 +10572,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K156" t="inlineStr"/>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L156" t="inlineStr">
         <is>
           <t>USD</t>
@@ -10017,7 +10637,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K157" t="inlineStr"/>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L157" t="inlineStr">
         <is>
           <t>USD</t>
@@ -10078,7 +10702,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K158" t="inlineStr"/>
+      <c r="K158" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L158" t="inlineStr">
         <is>
           <t>USD</t>
@@ -10139,7 +10767,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K159" t="inlineStr"/>
+      <c r="K159" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L159" t="inlineStr">
         <is>
           <t>USD</t>
@@ -10200,7 +10832,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K160" t="inlineStr"/>
+      <c r="K160" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L160" t="inlineStr">
         <is>
           <t>USD</t>
@@ -10261,7 +10897,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K161" t="inlineStr"/>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L161" t="inlineStr">
         <is>
           <t>USD</t>
@@ -10322,7 +10962,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K162" t="inlineStr"/>
+      <c r="K162" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L162" t="inlineStr">
         <is>
           <t>USD</t>
@@ -10383,7 +11027,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K163" t="inlineStr"/>
+      <c r="K163" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L163" t="inlineStr">
         <is>
           <t>USD</t>
@@ -10444,7 +11092,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K164" t="inlineStr"/>
+      <c r="K164" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L164" t="inlineStr">
         <is>
           <t>USD</t>
@@ -10505,7 +11157,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K165" t="inlineStr"/>
+      <c r="K165" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L165" t="inlineStr">
         <is>
           <t>USD</t>
@@ -10566,7 +11222,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K166" t="inlineStr"/>
+      <c r="K166" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L166" t="inlineStr">
         <is>
           <t>USD</t>
@@ -10627,7 +11287,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K167" t="inlineStr"/>
+      <c r="K167" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L167" t="inlineStr">
         <is>
           <t>USD</t>
@@ -10688,7 +11352,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K168" t="inlineStr"/>
+      <c r="K168" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L168" t="inlineStr">
         <is>
           <t>USD</t>
@@ -10749,7 +11417,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K169" t="inlineStr"/>
+      <c r="K169" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L169" t="inlineStr">
         <is>
           <t>USD</t>
@@ -10810,7 +11482,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K170" t="inlineStr"/>
+      <c r="K170" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L170" t="inlineStr">
         <is>
           <t>USD</t>
@@ -10871,7 +11547,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K171" t="inlineStr"/>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L171" t="inlineStr">
         <is>
           <t>USD</t>
@@ -10932,7 +11612,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K172" t="inlineStr"/>
+      <c r="K172" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L172" t="inlineStr">
         <is>
           <t>USD</t>
@@ -10993,7 +11677,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K173" t="inlineStr"/>
+      <c r="K173" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L173" t="inlineStr">
         <is>
           <t>USD</t>
@@ -11054,7 +11742,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K174" t="inlineStr"/>
+      <c r="K174" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L174" t="inlineStr">
         <is>
           <t>USD</t>
@@ -11115,7 +11807,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K175" t="inlineStr"/>
+      <c r="K175" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L175" t="inlineStr">
         <is>
           <t>USD</t>
@@ -11176,7 +11872,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K176" t="inlineStr"/>
+      <c r="K176" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L176" t="inlineStr">
         <is>
           <t>USD</t>
@@ -11237,7 +11937,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K177" t="inlineStr"/>
+      <c r="K177" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L177" t="inlineStr">
         <is>
           <t>USD</t>
@@ -11298,7 +12002,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K178" t="inlineStr"/>
+      <c r="K178" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L178" t="inlineStr">
         <is>
           <t>USD</t>
@@ -11359,7 +12067,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K179" t="inlineStr"/>
+      <c r="K179" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L179" t="inlineStr">
         <is>
           <t>USD</t>
@@ -11420,7 +12132,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K180" t="inlineStr"/>
+      <c r="K180" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L180" t="inlineStr">
         <is>
           <t>USD</t>
@@ -11481,7 +12197,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K181" t="inlineStr"/>
+      <c r="K181" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L181" t="inlineStr">
         <is>
           <t>USD</t>
@@ -11542,7 +12262,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K182" t="inlineStr"/>
+      <c r="K182" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L182" t="inlineStr">
         <is>
           <t>USD</t>
@@ -11603,7 +12327,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K183" t="inlineStr"/>
+      <c r="K183" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L183" t="inlineStr">
         <is>
           <t>USD</t>
@@ -11664,7 +12392,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K184" t="inlineStr"/>
+      <c r="K184" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L184" t="inlineStr">
         <is>
           <t>USD</t>
@@ -11725,7 +12457,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K185" t="inlineStr"/>
+      <c r="K185" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L185" t="inlineStr">
         <is>
           <t>USD</t>
@@ -11786,7 +12522,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K186" t="inlineStr"/>
+      <c r="K186" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L186" t="inlineStr">
         <is>
           <t>USD</t>
@@ -11847,7 +12587,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K187" t="inlineStr"/>
+      <c r="K187" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L187" t="inlineStr">
         <is>
           <t>USD</t>
@@ -11908,7 +12652,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K188" t="inlineStr"/>
+      <c r="K188" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L188" t="inlineStr">
         <is>
           <t>USD</t>
@@ -11969,7 +12717,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K189" t="inlineStr"/>
+      <c r="K189" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L189" t="inlineStr">
         <is>
           <t>USD</t>
@@ -12030,7 +12782,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K190" t="inlineStr"/>
+      <c r="K190" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L190" t="inlineStr">
         <is>
           <t>USD</t>
@@ -12091,7 +12847,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K191" t="inlineStr"/>
+      <c r="K191" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L191" t="inlineStr">
         <is>
           <t>USD</t>
@@ -12152,7 +12912,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K192" t="inlineStr"/>
+      <c r="K192" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L192" t="inlineStr">
         <is>
           <t>USD</t>
@@ -12213,7 +12977,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K193" t="inlineStr"/>
+      <c r="K193" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L193" t="inlineStr">
         <is>
           <t>USD</t>
@@ -12274,7 +13042,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K194" t="inlineStr"/>
+      <c r="K194" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L194" t="inlineStr">
         <is>
           <t>USD</t>
@@ -12335,7 +13107,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K195" t="inlineStr"/>
+      <c r="K195" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L195" t="inlineStr">
         <is>
           <t>USD</t>
@@ -12396,7 +13172,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K196" t="inlineStr"/>
+      <c r="K196" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L196" t="inlineStr">
         <is>
           <t>USD</t>
@@ -12457,7 +13237,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K197" t="inlineStr"/>
+      <c r="K197" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L197" t="inlineStr">
         <is>
           <t>USD</t>
@@ -12518,7 +13302,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K198" t="inlineStr"/>
+      <c r="K198" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L198" t="inlineStr">
         <is>
           <t>USD</t>
@@ -12579,7 +13367,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K199" t="inlineStr"/>
+      <c r="K199" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L199" t="inlineStr">
         <is>
           <t>USD</t>
@@ -12640,7 +13432,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K200" t="inlineStr"/>
+      <c r="K200" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L200" t="inlineStr">
         <is>
           <t>USD</t>
@@ -12701,7 +13497,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K201" t="inlineStr"/>
+      <c r="K201" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L201" t="inlineStr">
         <is>
           <t>USD</t>
@@ -12762,7 +13562,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K202" t="inlineStr"/>
+      <c r="K202" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L202" t="inlineStr">
         <is>
           <t>USD</t>
@@ -12823,7 +13627,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K203" t="inlineStr"/>
+      <c r="K203" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L203" t="inlineStr">
         <is>
           <t>USD</t>
@@ -12884,7 +13692,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K204" t="inlineStr"/>
+      <c r="K204" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L204" t="inlineStr">
         <is>
           <t>USD</t>
@@ -12945,7 +13757,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K205" t="inlineStr"/>
+      <c r="K205" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L205" t="inlineStr">
         <is>
           <t>USD</t>
@@ -13006,7 +13822,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K206" t="inlineStr"/>
+      <c r="K206" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L206" t="inlineStr">
         <is>
           <t>USD</t>
@@ -13067,7 +13887,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K207" t="inlineStr"/>
+      <c r="K207" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L207" t="inlineStr">
         <is>
           <t>USD</t>
@@ -13128,7 +13952,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K208" t="inlineStr"/>
+      <c r="K208" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L208" t="inlineStr">
         <is>
           <t>USD</t>
@@ -13189,7 +14017,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K209" t="inlineStr"/>
+      <c r="K209" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L209" t="inlineStr">
         <is>
           <t>USD</t>
@@ -13250,7 +14082,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K210" t="inlineStr"/>
+      <c r="K210" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L210" t="inlineStr">
         <is>
           <t>USD</t>
@@ -13311,7 +14147,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K211" t="inlineStr"/>
+      <c r="K211" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L211" t="inlineStr">
         <is>
           <t>USD</t>
@@ -13372,7 +14212,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K212" t="inlineStr"/>
+      <c r="K212" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L212" t="inlineStr">
         <is>
           <t>USD</t>
@@ -13433,7 +14277,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K213" t="inlineStr"/>
+      <c r="K213" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L213" t="inlineStr">
         <is>
           <t>USD</t>
@@ -13494,7 +14342,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K214" t="inlineStr"/>
+      <c r="K214" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L214" t="inlineStr">
         <is>
           <t>USD</t>
@@ -13555,7 +14407,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K215" t="inlineStr"/>
+      <c r="K215" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L215" t="inlineStr">
         <is>
           <t>USD</t>
@@ -13616,7 +14472,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K216" t="inlineStr"/>
+      <c r="K216" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L216" t="inlineStr">
         <is>
           <t>USD</t>
@@ -13677,7 +14537,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K217" t="inlineStr"/>
+      <c r="K217" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L217" t="inlineStr">
         <is>
           <t>USD</t>
@@ -13738,7 +14602,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K218" t="inlineStr"/>
+      <c r="K218" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L218" t="inlineStr">
         <is>
           <t>USD</t>
@@ -13799,7 +14667,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K219" t="inlineStr"/>
+      <c r="K219" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L219" t="inlineStr">
         <is>
           <t>USD</t>
@@ -13860,7 +14732,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K220" t="inlineStr"/>
+      <c r="K220" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L220" t="inlineStr">
         <is>
           <t>USD</t>
@@ -13921,7 +14797,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K221" t="inlineStr"/>
+      <c r="K221" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L221" t="inlineStr">
         <is>
           <t>USD</t>
@@ -13982,7 +14862,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K222" t="inlineStr"/>
+      <c r="K222" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L222" t="inlineStr">
         <is>
           <t>USD</t>
@@ -14043,7 +14927,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K223" t="inlineStr"/>
+      <c r="K223" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L223" t="inlineStr">
         <is>
           <t>USD</t>
@@ -14104,7 +14992,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K224" t="inlineStr"/>
+      <c r="K224" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L224" t="inlineStr">
         <is>
           <t>USD</t>
@@ -14165,7 +15057,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K225" t="inlineStr"/>
+      <c r="K225" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L225" t="inlineStr">
         <is>
           <t>USD</t>
@@ -14226,7 +15122,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K226" t="inlineStr"/>
+      <c r="K226" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L226" t="inlineStr">
         <is>
           <t>USD</t>
@@ -14287,7 +15187,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K227" t="inlineStr"/>
+      <c r="K227" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L227" t="inlineStr">
         <is>
           <t>USD</t>
@@ -14348,7 +15252,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K228" t="inlineStr"/>
+      <c r="K228" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L228" t="inlineStr">
         <is>
           <t>USD</t>
@@ -14409,7 +15317,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K229" t="inlineStr"/>
+      <c r="K229" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L229" t="inlineStr">
         <is>
           <t>USD</t>
@@ -14470,7 +15382,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K230" t="inlineStr"/>
+      <c r="K230" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L230" t="inlineStr">
         <is>
           <t>USD</t>
@@ -14531,7 +15447,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K231" t="inlineStr"/>
+      <c r="K231" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L231" t="inlineStr">
         <is>
           <t>USD</t>
@@ -14592,7 +15512,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K232" t="inlineStr"/>
+      <c r="K232" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L232" t="inlineStr">
         <is>
           <t>USD</t>
@@ -14653,7 +15577,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K233" t="inlineStr"/>
+      <c r="K233" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L233" t="inlineStr">
         <is>
           <t>USD</t>
@@ -14714,7 +15642,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K234" t="inlineStr"/>
+      <c r="K234" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L234" t="inlineStr">
         <is>
           <t>USD</t>
@@ -14775,7 +15707,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K235" t="inlineStr"/>
+      <c r="K235" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L235" t="inlineStr">
         <is>
           <t>USD</t>
@@ -14836,7 +15772,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K236" t="inlineStr"/>
+      <c r="K236" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L236" t="inlineStr">
         <is>
           <t>USD</t>
@@ -14897,7 +15837,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K237" t="inlineStr"/>
+      <c r="K237" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L237" t="inlineStr">
         <is>
           <t>USD</t>
@@ -14958,7 +15902,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K238" t="inlineStr"/>
+      <c r="K238" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L238" t="inlineStr">
         <is>
           <t>USD</t>
@@ -15019,7 +15967,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K239" t="inlineStr"/>
+      <c r="K239" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L239" t="inlineStr">
         <is>
           <t>USD</t>
@@ -15080,7 +16032,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K240" t="inlineStr"/>
+      <c r="K240" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L240" t="inlineStr">
         <is>
           <t>USD</t>
@@ -15141,7 +16097,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K241" t="inlineStr"/>
+      <c r="K241" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L241" t="inlineStr">
         <is>
           <t>USD</t>
@@ -15202,7 +16162,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K242" t="inlineStr"/>
+      <c r="K242" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L242" t="inlineStr">
         <is>
           <t>USD</t>
@@ -15263,7 +16227,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K243" t="inlineStr"/>
+      <c r="K243" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L243" t="inlineStr">
         <is>
           <t>USD</t>
@@ -15324,7 +16292,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K244" t="inlineStr"/>
+      <c r="K244" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L244" t="inlineStr">
         <is>
           <t>USD</t>
@@ -15385,7 +16357,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K245" t="inlineStr"/>
+      <c r="K245" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L245" t="inlineStr">
         <is>
           <t>USD</t>
@@ -15446,7 +16422,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K246" t="inlineStr"/>
+      <c r="K246" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L246" t="inlineStr">
         <is>
           <t>USD</t>
@@ -15507,7 +16487,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K247" t="inlineStr"/>
+      <c r="K247" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L247" t="inlineStr">
         <is>
           <t>USD</t>
@@ -15568,7 +16552,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K248" t="inlineStr"/>
+      <c r="K248" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L248" t="inlineStr">
         <is>
           <t>USD</t>
@@ -15629,7 +16617,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K249" t="inlineStr"/>
+      <c r="K249" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L249" t="inlineStr">
         <is>
           <t>USD</t>
@@ -15690,7 +16682,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K250" t="inlineStr"/>
+      <c r="K250" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L250" t="inlineStr">
         <is>
           <t>USD</t>
@@ -15751,7 +16747,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K251" t="inlineStr"/>
+      <c r="K251" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L251" t="inlineStr">
         <is>
           <t>USD</t>
@@ -15812,7 +16812,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K252" t="inlineStr"/>
+      <c r="K252" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L252" t="inlineStr">
         <is>
           <t>USD</t>
@@ -15873,7 +16877,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K253" t="inlineStr"/>
+      <c r="K253" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L253" t="inlineStr">
         <is>
           <t>USD</t>
@@ -15934,7 +16942,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K254" t="inlineStr"/>
+      <c r="K254" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L254" t="inlineStr">
         <is>
           <t>USD</t>
@@ -15995,7 +17007,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K255" t="inlineStr"/>
+      <c r="K255" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L255" t="inlineStr">
         <is>
           <t>USD</t>
@@ -16056,7 +17072,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K256" t="inlineStr"/>
+      <c r="K256" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L256" t="inlineStr">
         <is>
           <t>USD</t>
@@ -16117,7 +17137,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K257" t="inlineStr"/>
+      <c r="K257" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L257" t="inlineStr">
         <is>
           <t>USD</t>
@@ -16178,7 +17202,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K258" t="inlineStr"/>
+      <c r="K258" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L258" t="inlineStr">
         <is>
           <t>USD</t>
@@ -16239,7 +17267,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K259" t="inlineStr"/>
+      <c r="K259" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L259" t="inlineStr">
         <is>
           <t>USD</t>
@@ -16300,7 +17332,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K260" t="inlineStr"/>
+      <c r="K260" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L260" t="inlineStr">
         <is>
           <t>USD</t>
@@ -16361,7 +17397,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K261" t="inlineStr"/>
+      <c r="K261" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L261" t="inlineStr">
         <is>
           <t>USD</t>
@@ -16422,7 +17462,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K262" t="inlineStr"/>
+      <c r="K262" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L262" t="inlineStr">
         <is>
           <t>USD</t>
@@ -16483,7 +17527,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K263" t="inlineStr"/>
+      <c r="K263" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L263" t="inlineStr">
         <is>
           <t>USD</t>
@@ -16544,7 +17592,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K264" t="inlineStr"/>
+      <c r="K264" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L264" t="inlineStr">
         <is>
           <t>USD</t>
@@ -16605,7 +17657,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K265" t="inlineStr"/>
+      <c r="K265" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L265" t="inlineStr">
         <is>
           <t>USD</t>
@@ -16666,7 +17722,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K266" t="inlineStr"/>
+      <c r="K266" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L266" t="inlineStr">
         <is>
           <t>USD</t>
@@ -16727,7 +17787,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K267" t="inlineStr"/>
+      <c r="K267" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L267" t="inlineStr">
         <is>
           <t>USD</t>
@@ -16788,7 +17852,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K268" t="inlineStr"/>
+      <c r="K268" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L268" t="inlineStr">
         <is>
           <t>USD</t>
@@ -16849,7 +17917,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K269" t="inlineStr"/>
+      <c r="K269" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L269" t="inlineStr">
         <is>
           <t>USD</t>
@@ -16910,7 +17982,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K270" t="inlineStr"/>
+      <c r="K270" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L270" t="inlineStr">
         <is>
           <t>USD</t>
@@ -16971,7 +18047,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K271" t="inlineStr"/>
+      <c r="K271" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L271" t="inlineStr">
         <is>
           <t>USD</t>
@@ -17032,7 +18112,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K272" t="inlineStr"/>
+      <c r="K272" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L272" t="inlineStr">
         <is>
           <t>USD</t>
@@ -17093,7 +18177,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K273" t="inlineStr"/>
+      <c r="K273" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L273" t="inlineStr">
         <is>
           <t>USD</t>
@@ -17154,7 +18242,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K274" t="inlineStr"/>
+      <c r="K274" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L274" t="inlineStr">
         <is>
           <t>USD</t>
@@ -17215,7 +18307,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K275" t="inlineStr"/>
+      <c r="K275" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L275" t="inlineStr">
         <is>
           <t>USD</t>
@@ -17276,7 +18372,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K276" t="inlineStr"/>
+      <c r="K276" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L276" t="inlineStr">
         <is>
           <t>USD</t>
@@ -17337,7 +18437,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K277" t="inlineStr"/>
+      <c r="K277" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L277" t="inlineStr">
         <is>
           <t>USD</t>
@@ -17398,7 +18502,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K278" t="inlineStr"/>
+      <c r="K278" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L278" t="inlineStr">
         <is>
           <t>USD</t>
@@ -17459,7 +18567,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K279" t="inlineStr"/>
+      <c r="K279" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L279" t="inlineStr">
         <is>
           <t>USD</t>
@@ -17520,7 +18632,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K280" t="inlineStr"/>
+      <c r="K280" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L280" t="inlineStr">
         <is>
           <t>USD</t>
@@ -17581,7 +18697,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K281" t="inlineStr"/>
+      <c r="K281" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L281" t="inlineStr">
         <is>
           <t>USD</t>
@@ -17642,7 +18762,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K282" t="inlineStr"/>
+      <c r="K282" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L282" t="inlineStr">
         <is>
           <t>USD</t>
@@ -17703,7 +18827,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K283" t="inlineStr"/>
+      <c r="K283" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L283" t="inlineStr">
         <is>
           <t>USD</t>
@@ -17764,7 +18892,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K284" t="inlineStr"/>
+      <c r="K284" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L284" t="inlineStr">
         <is>
           <t>USD</t>
@@ -17825,7 +18957,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K285" t="inlineStr"/>
+      <c r="K285" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L285" t="inlineStr">
         <is>
           <t>USD</t>
@@ -17886,7 +19022,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K286" t="inlineStr"/>
+      <c r="K286" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L286" t="inlineStr">
         <is>
           <t>USD</t>
@@ -17947,7 +19087,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K287" t="inlineStr"/>
+      <c r="K287" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L287" t="inlineStr">
         <is>
           <t>USD</t>
@@ -18008,7 +19152,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K288" t="inlineStr"/>
+      <c r="K288" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L288" t="inlineStr">
         <is>
           <t>USD</t>
@@ -18069,7 +19217,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K289" t="inlineStr"/>
+      <c r="K289" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L289" t="inlineStr">
         <is>
           <t>USD</t>
@@ -18130,7 +19282,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K290" t="inlineStr"/>
+      <c r="K290" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L290" t="inlineStr">
         <is>
           <t>USD</t>
@@ -18191,7 +19347,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K291" t="inlineStr"/>
+      <c r="K291" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L291" t="inlineStr">
         <is>
           <t>USD</t>
@@ -18252,7 +19412,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K292" t="inlineStr"/>
+      <c r="K292" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L292" t="inlineStr">
         <is>
           <t>USD</t>
@@ -18313,7 +19477,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K293" t="inlineStr"/>
+      <c r="K293" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L293" t="inlineStr">
         <is>
           <t>USD</t>
@@ -18374,7 +19542,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K294" t="inlineStr"/>
+      <c r="K294" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L294" t="inlineStr">
         <is>
           <t>USD</t>
@@ -18435,7 +19607,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K295" t="inlineStr"/>
+      <c r="K295" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L295" t="inlineStr">
         <is>
           <t>USD</t>
@@ -18496,7 +19672,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K296" t="inlineStr"/>
+      <c r="K296" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L296" t="inlineStr">
         <is>
           <t>USD</t>
@@ -18557,7 +19737,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K297" t="inlineStr"/>
+      <c r="K297" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L297" t="inlineStr">
         <is>
           <t>USD</t>
@@ -18618,7 +19802,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K298" t="inlineStr"/>
+      <c r="K298" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L298" t="inlineStr">
         <is>
           <t>USD</t>
@@ -18679,7 +19867,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K299" t="inlineStr"/>
+      <c r="K299" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L299" t="inlineStr">
         <is>
           <t>USD</t>
@@ -18740,7 +19932,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K300" t="inlineStr"/>
+      <c r="K300" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L300" t="inlineStr">
         <is>
           <t>USD</t>
@@ -18801,7 +19997,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K301" t="inlineStr"/>
+      <c r="K301" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L301" t="inlineStr">
         <is>
           <t>USD</t>
@@ -18862,7 +20062,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K302" t="inlineStr"/>
+      <c r="K302" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L302" t="inlineStr">
         <is>
           <t>USD</t>
@@ -18923,7 +20127,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K303" t="inlineStr"/>
+      <c r="K303" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L303" t="inlineStr">
         <is>
           <t>USD</t>
@@ -18984,7 +20192,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K304" t="inlineStr"/>
+      <c r="K304" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L304" t="inlineStr">
         <is>
           <t>USD</t>
@@ -19045,7 +20257,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K305" t="inlineStr"/>
+      <c r="K305" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L305" t="inlineStr">
         <is>
           <t>USD</t>
@@ -19106,7 +20322,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K306" t="inlineStr"/>
+      <c r="K306" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L306" t="inlineStr">
         <is>
           <t>USD</t>
@@ -19167,7 +20387,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K307" t="inlineStr"/>
+      <c r="K307" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L307" t="inlineStr">
         <is>
           <t>USD</t>
@@ -19228,7 +20452,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K308" t="inlineStr"/>
+      <c r="K308" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L308" t="inlineStr">
         <is>
           <t>USD</t>
@@ -19289,7 +20517,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K309" t="inlineStr"/>
+      <c r="K309" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L309" t="inlineStr">
         <is>
           <t>USD</t>
@@ -19350,7 +20582,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K310" t="inlineStr"/>
+      <c r="K310" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L310" t="inlineStr">
         <is>
           <t>USD</t>
@@ -19411,7 +20647,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K311" t="inlineStr"/>
+      <c r="K311" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L311" t="inlineStr">
         <is>
           <t>USD</t>
@@ -19472,7 +20712,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K312" t="inlineStr"/>
+      <c r="K312" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L312" t="inlineStr">
         <is>
           <t>USD</t>
@@ -19533,7 +20777,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K313" t="inlineStr"/>
+      <c r="K313" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L313" t="inlineStr">
         <is>
           <t>USD</t>
@@ -19594,7 +20842,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K314" t="inlineStr"/>
+      <c r="K314" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L314" t="inlineStr">
         <is>
           <t>USD</t>
@@ -19655,7 +20907,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K315" t="inlineStr"/>
+      <c r="K315" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L315" t="inlineStr">
         <is>
           <t>USD</t>
@@ -19716,7 +20972,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K316" t="inlineStr"/>
+      <c r="K316" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L316" t="inlineStr">
         <is>
           <t>USD</t>
@@ -19777,7 +21037,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K317" t="inlineStr"/>
+      <c r="K317" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L317" t="inlineStr">
         <is>
           <t>USD</t>
@@ -19838,7 +21102,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K318" t="inlineStr"/>
+      <c r="K318" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L318" t="inlineStr">
         <is>
           <t>USD</t>
@@ -19899,7 +21167,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K319" t="inlineStr"/>
+      <c r="K319" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L319" t="inlineStr">
         <is>
           <t>USD</t>
@@ -19960,7 +21232,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K320" t="inlineStr"/>
+      <c r="K320" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L320" t="inlineStr">
         <is>
           <t>USD</t>
@@ -20021,7 +21297,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K321" t="inlineStr"/>
+      <c r="K321" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L321" t="inlineStr">
         <is>
           <t>USD</t>
@@ -20082,7 +21362,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K322" t="inlineStr"/>
+      <c r="K322" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L322" t="inlineStr">
         <is>
           <t>USD</t>
@@ -20143,7 +21427,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K323" t="inlineStr"/>
+      <c r="K323" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L323" t="inlineStr">
         <is>
           <t>USD</t>
@@ -20204,7 +21492,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K324" t="inlineStr"/>
+      <c r="K324" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L324" t="inlineStr">
         <is>
           <t>USD</t>
@@ -20265,7 +21557,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K325" t="inlineStr"/>
+      <c r="K325" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L325" t="inlineStr">
         <is>
           <t>USD</t>
@@ -20326,7 +21622,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K326" t="inlineStr"/>
+      <c r="K326" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L326" t="inlineStr">
         <is>
           <t>USD</t>
@@ -20387,7 +21687,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K327" t="inlineStr"/>
+      <c r="K327" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L327" t="inlineStr">
         <is>
           <t>USD</t>
@@ -20448,7 +21752,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K328" t="inlineStr"/>
+      <c r="K328" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L328" t="inlineStr">
         <is>
           <t>USD</t>
@@ -20509,7 +21817,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K329" t="inlineStr"/>
+      <c r="K329" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L329" t="inlineStr">
         <is>
           <t>USD</t>
@@ -20570,7 +21882,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K330" t="inlineStr"/>
+      <c r="K330" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L330" t="inlineStr">
         <is>
           <t>USD</t>
@@ -20631,7 +21947,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K331" t="inlineStr"/>
+      <c r="K331" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L331" t="inlineStr">
         <is>
           <t>USD</t>
@@ -20692,7 +22012,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K332" t="inlineStr"/>
+      <c r="K332" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L332" t="inlineStr">
         <is>
           <t>USD</t>
@@ -20753,7 +22077,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K333" t="inlineStr"/>
+      <c r="K333" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L333" t="inlineStr">
         <is>
           <t>USD</t>
@@ -20814,7 +22142,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K334" t="inlineStr"/>
+      <c r="K334" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L334" t="inlineStr">
         <is>
           <t>USD</t>
@@ -20875,7 +22207,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K335" t="inlineStr"/>
+      <c r="K335" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L335" t="inlineStr">
         <is>
           <t>USD</t>
@@ -20936,7 +22272,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K336" t="inlineStr"/>
+      <c r="K336" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L336" t="inlineStr">
         <is>
           <t>USD</t>
@@ -20997,7 +22337,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K337" t="inlineStr"/>
+      <c r="K337" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L337" t="inlineStr">
         <is>
           <t>USD</t>
@@ -21058,7 +22402,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K338" t="inlineStr"/>
+      <c r="K338" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L338" t="inlineStr">
         <is>
           <t>USD</t>
@@ -21119,7 +22467,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K339" t="inlineStr"/>
+      <c r="K339" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L339" t="inlineStr">
         <is>
           <t>USD</t>
@@ -21180,7 +22532,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K340" t="inlineStr"/>
+      <c r="K340" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L340" t="inlineStr">
         <is>
           <t>USD</t>
@@ -21241,7 +22597,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K341" t="inlineStr"/>
+      <c r="K341" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L341" t="inlineStr">
         <is>
           <t>USD</t>
@@ -21302,7 +22662,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K342" t="inlineStr"/>
+      <c r="K342" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L342" t="inlineStr">
         <is>
           <t>USD</t>
@@ -21363,7 +22727,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K343" t="inlineStr"/>
+      <c r="K343" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L343" t="inlineStr">
         <is>
           <t>USD</t>
@@ -21424,7 +22792,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K344" t="inlineStr"/>
+      <c r="K344" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L344" t="inlineStr">
         <is>
           <t>USD</t>
@@ -21485,7 +22857,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K345" t="inlineStr"/>
+      <c r="K345" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L345" t="inlineStr">
         <is>
           <t>USD</t>
@@ -21546,7 +22922,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K346" t="inlineStr"/>
+      <c r="K346" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L346" t="inlineStr">
         <is>
           <t>USD</t>
@@ -21607,7 +22987,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K347" t="inlineStr"/>
+      <c r="K347" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L347" t="inlineStr">
         <is>
           <t>USD</t>
@@ -21668,7 +23052,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K348" t="inlineStr"/>
+      <c r="K348" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L348" t="inlineStr">
         <is>
           <t>USD</t>
@@ -21729,7 +23117,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K349" t="inlineStr"/>
+      <c r="K349" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L349" t="inlineStr">
         <is>
           <t>USD</t>
@@ -21790,7 +23182,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K350" t="inlineStr"/>
+      <c r="K350" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L350" t="inlineStr">
         <is>
           <t>USD</t>
@@ -21851,7 +23247,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K351" t="inlineStr"/>
+      <c r="K351" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L351" t="inlineStr">
         <is>
           <t>USD</t>
@@ -21912,7 +23312,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K352" t="inlineStr"/>
+      <c r="K352" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L352" t="inlineStr">
         <is>
           <t>USD</t>
@@ -21973,7 +23377,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K353" t="inlineStr"/>
+      <c r="K353" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L353" t="inlineStr">
         <is>
           <t>USD</t>
@@ -22034,7 +23442,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K354" t="inlineStr"/>
+      <c r="K354" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L354" t="inlineStr">
         <is>
           <t>USD</t>
@@ -22095,7 +23507,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K355" t="inlineStr"/>
+      <c r="K355" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L355" t="inlineStr">
         <is>
           <t>USD</t>
@@ -22156,7 +23572,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K356" t="inlineStr"/>
+      <c r="K356" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L356" t="inlineStr">
         <is>
           <t>USD</t>
@@ -22217,7 +23637,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K357" t="inlineStr"/>
+      <c r="K357" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L357" t="inlineStr">
         <is>
           <t>USD</t>
@@ -22278,7 +23702,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K358" t="inlineStr"/>
+      <c r="K358" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L358" t="inlineStr">
         <is>
           <t>USD</t>
@@ -22339,7 +23767,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K359" t="inlineStr"/>
+      <c r="K359" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L359" t="inlineStr">
         <is>
           <t>USD</t>
@@ -22400,7 +23832,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K360" t="inlineStr"/>
+      <c r="K360" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L360" t="inlineStr">
         <is>
           <t>USD</t>
@@ -22461,7 +23897,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K361" t="inlineStr"/>
+      <c r="K361" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L361" t="inlineStr">
         <is>
           <t>USD</t>
@@ -22522,7 +23962,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K362" t="inlineStr"/>
+      <c r="K362" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L362" t="inlineStr">
         <is>
           <t>USD</t>
@@ -22583,7 +24027,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K363" t="inlineStr"/>
+      <c r="K363" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L363" t="inlineStr">
         <is>
           <t>USD</t>
@@ -22644,7 +24092,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K364" t="inlineStr"/>
+      <c r="K364" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L364" t="inlineStr">
         <is>
           <t>USD</t>
@@ -22705,7 +24157,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K365" t="inlineStr"/>
+      <c r="K365" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L365" t="inlineStr">
         <is>
           <t>USD</t>
@@ -22766,7 +24222,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K366" t="inlineStr"/>
+      <c r="K366" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L366" t="inlineStr">
         <is>
           <t>USD</t>
@@ -22827,7 +24287,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K367" t="inlineStr"/>
+      <c r="K367" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L367" t="inlineStr">
         <is>
           <t>USD</t>
@@ -22888,7 +24352,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K368" t="inlineStr"/>
+      <c r="K368" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L368" t="inlineStr">
         <is>
           <t>USD</t>
@@ -22949,7 +24417,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K369" t="inlineStr"/>
+      <c r="K369" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L369" t="inlineStr">
         <is>
           <t>USD</t>
@@ -23010,7 +24482,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K370" t="inlineStr"/>
+      <c r="K370" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L370" t="inlineStr">
         <is>
           <t>USD</t>
@@ -23071,7 +24547,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K371" t="inlineStr"/>
+      <c r="K371" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L371" t="inlineStr">
         <is>
           <t>USD</t>
@@ -23132,7 +24612,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K372" t="inlineStr"/>
+      <c r="K372" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L372" t="inlineStr">
         <is>
           <t>USD</t>
@@ -23193,7 +24677,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K373" t="inlineStr"/>
+      <c r="K373" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L373" t="inlineStr">
         <is>
           <t>USD</t>
@@ -23254,7 +24742,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K374" t="inlineStr"/>
+      <c r="K374" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L374" t="inlineStr">
         <is>
           <t>USD</t>
@@ -23315,7 +24807,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K375" t="inlineStr"/>
+      <c r="K375" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L375" t="inlineStr">
         <is>
           <t>USD</t>
@@ -23376,7 +24872,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K376" t="inlineStr"/>
+      <c r="K376" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L376" t="inlineStr">
         <is>
           <t>USD</t>
@@ -23437,7 +24937,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K377" t="inlineStr"/>
+      <c r="K377" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L377" t="inlineStr">
         <is>
           <t>USD</t>
@@ -23498,7 +25002,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K378" t="inlineStr"/>
+      <c r="K378" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L378" t="inlineStr">
         <is>
           <t>USD</t>
@@ -23559,7 +25067,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K379" t="inlineStr"/>
+      <c r="K379" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L379" t="inlineStr">
         <is>
           <t>USD</t>
@@ -23620,7 +25132,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K380" t="inlineStr"/>
+      <c r="K380" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L380" t="inlineStr">
         <is>
           <t>USD</t>
@@ -23681,7 +25197,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K381" t="inlineStr"/>
+      <c r="K381" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L381" t="inlineStr">
         <is>
           <t>USD</t>
@@ -23742,7 +25262,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K382" t="inlineStr"/>
+      <c r="K382" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L382" t="inlineStr">
         <is>
           <t>USD</t>
@@ -23803,7 +25327,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K383" t="inlineStr"/>
+      <c r="K383" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L383" t="inlineStr">
         <is>
           <t>USD</t>
@@ -23864,7 +25392,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K384" t="inlineStr"/>
+      <c r="K384" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L384" t="inlineStr">
         <is>
           <t>USD</t>
@@ -23925,7 +25457,11 @@
           <t>96.781.350-8</t>
         </is>
       </c>
-      <c r="K385" t="inlineStr"/>
+      <c r="K385" t="inlineStr">
+        <is>
+          <t>Metropolitana</t>
+        </is>
+      </c>
       <c r="L385" t="inlineStr">
         <is>
           <t>USD</t>

</xml_diff>